<commit_message>
Architettura dati: scheduler giornaliero + cache su disco
- Rimuove pulsante Carica Dati: i dati si caricano automaticamente da
  market_data.pkl all'avvio; APScheduler aggiorna ogni giorno alle 18:30
- Aggiunge pulsante Aggiorna per refresh manuale
- Ottimizza grafici: CVaR vectorizzato, filtro IR su tail-only
- Aggiunge supporto proxy/User-Agent per ambienti cloud (Render)
- Aggiorna TARBIUTH.xlsx con nomi asset abbreviati
- Aggiunge apscheduler a requirements.txt

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TARBIUTH.xlsx
+++ b/TARBIUTH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookpro/Downloads/andcappe_zip/Dashboard/SITO_WEB/Sito personale/portafoglio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9449700B-A48E-2D49-BEB2-DC2C96EFB068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{76750A06-1780-A740-A3CE-CB2DF706D97E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4380" yWindow="20" windowWidth="24420" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7568" uniqueCount="2729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7566" uniqueCount="2749">
   <si>
     <t>Simbolo</t>
   </si>
@@ -8476,28 +8476,88 @@
     <t>CSBGE3.MI</t>
   </si>
   <si>
-    <t>iShares VII PLC - iShares € Govt Bond 1-3yr</t>
-  </si>
-  <si>
-    <t>iShares VII PLC - iShares € Govt Bond 3-7yr</t>
-  </si>
-  <si>
     <t>SXRQ.DE</t>
   </si>
   <si>
-    <t>iShares VII PLC - iShares € Govt Bond 7-10yr</t>
-  </si>
-  <si>
     <t>XEIN.DE</t>
   </si>
   <si>
-    <t>Xtrackers II Global Inflation-Linked Bond UCITS ETF 1C - EUR Hedged</t>
-  </si>
-  <si>
-    <t>State Street SPDR FTSE Global Convertible Bond hdg</t>
-  </si>
-  <si>
     <t>Alternative</t>
+  </si>
+  <si>
+    <t>Az. ACWI</t>
+  </si>
+  <si>
+    <t>Az.USA Nasdaq100</t>
+  </si>
+  <si>
+    <t>Az. USA SP500</t>
+  </si>
+  <si>
+    <t>Az. USA Growth SP500</t>
+  </si>
+  <si>
+    <t>Az. USA Growth</t>
+  </si>
+  <si>
+    <t>Az.  USA Value SP500</t>
+  </si>
+  <si>
+    <t>Az USA Value Small Cap</t>
+  </si>
+  <si>
+    <t>Az. World Value Factor</t>
+  </si>
+  <si>
+    <t>Az EUROPA Value Small Cap</t>
+  </si>
+  <si>
+    <t>Az USA Small Cap Russell2000</t>
+  </si>
+  <si>
+    <t>Az. World</t>
+  </si>
+  <si>
+    <t>Az. Europe Stoxx 600</t>
+  </si>
+  <si>
+    <t>Az. Emerging Market</t>
+  </si>
+  <si>
+    <t>OB. Govt Bond 1-3yr</t>
+  </si>
+  <si>
+    <t>Ob. Govt Bond 3-7yr</t>
+  </si>
+  <si>
+    <t>Ob. Govt Bond 7-10yr</t>
+  </si>
+  <si>
+    <t>Ob. Corp Bond 1-3yr UCITS ETF</t>
+  </si>
+  <si>
+    <t>Ob. EUR Corporate Bond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ob. EUR High Yield Corporate Bond </t>
+  </si>
+  <si>
+    <t>Ob. Eurozone Infl-Linked Bond</t>
+  </si>
+  <si>
+    <t>Ob. Global Inflation-Linked Hedged</t>
+  </si>
+  <si>
+    <t>Ob. Global Convertible Bond hdg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gold </t>
+  </si>
+  <si>
+    <t>AZ. VANGUARD ACWI</t>
+  </si>
+  <si>
+    <t>Azionario ACWI Vanguard</t>
   </si>
 </sst>
 </file>
@@ -9138,23 +9198,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Arial Nova"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF232A31"/>
-      <name val="Arial Nova"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color theme="10"/>
-      <name val="Arial Nova"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF1F3864"/>
@@ -9191,6 +9234,23 @@
       <name val="Helvetica Neue"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="8"/>
+      <name val="Abadi"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF232A31"/>
+      <name val="Abadi"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color theme="10"/>
+      <name val="Abadi"/>
     </font>
   </fonts>
   <fills count="12">
@@ -9464,7 +9524,7 @@
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="26" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="240">
+  <cellXfs count="241">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -9770,14 +9830,27 @@
     <xf numFmtId="0" fontId="87" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="96" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="96" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="97" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="98" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="96" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="98" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="99" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="99" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="96" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="100" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="99" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="99" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="98" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="98" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="85" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -9789,27 +9862,17 @@
     <xf numFmtId="0" fontId="83" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="99" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="100" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="101" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="102" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="102" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="101" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="103" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="102" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="102" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="101" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="101" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="101" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="101" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="102" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="103" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="101" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -9818,7 +9881,7 @@
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
     <cellStyle name="Percentuale" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="12">
     <dxf>
       <font>
         <b val="0"/>
@@ -9830,11 +9893,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color indexed="8"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="major"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -9843,10 +9905,77 @@
         <outline val="0"/>
         <shadow val="0"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="major"/>
+        <sz val="9"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -9934,76 +10063,21 @@
         <vertAlign val="baseline"/>
         <sz val="10"/>
         <color indexed="8"/>
-        <name val="Arial Nova"/>
-        <scheme val="none"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="major"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color indexed="8"/>
-        <name val="Arial Nova"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <name val="Arial Nova"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <name val="Arial Nova"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <name val="Arial Nova"/>
-        <scheme val="none"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="major"/>
       </font>
     </dxf>
   </dxfs>
@@ -16189,26 +16263,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D26" totalsRowShown="0" dataDxfId="10">
-  <autoFilter ref="A1:D26" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D25" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:D25" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{12AF85F4-CF3E-1A44-9197-52CD700ECF69}" name="SIMBOLO" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{D2DEAFE7-7181-F841-96D9-E16F6CD58118}" name="DESCRIZIONE" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{036B7D95-54D0-CE4A-A97C-6EC741E876E4}" name="VALUTA" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{BC856CD8-BE7C-D246-AFFE-8A0458341DA0}" name="CLASSE" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{12AF85F4-CF3E-1A44-9197-52CD700ECF69}" name="SIMBOLO" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{D2DEAFE7-7181-F841-96D9-E16F6CD58118}" name="DESCRIZIONE" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{036B7D95-54D0-CE4A-A97C-6EC741E876E4}" name="VALUTA" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{BC856CD8-BE7C-D246-AFFE-8A0458341DA0}" name="CLASSE" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}" name="Tabella323" displayName="Tabella323" ref="A1:D53" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}" name="Tabella323" displayName="Tabella323" ref="A1:D53" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:D53" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{99BE53A6-82BE-7C4C-8EDB-FC2585DE7E29}" name="SIMBOLO" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{79CB9D70-57D7-004E-8DD2-11CA0A269F24}" name="DESCRIZIONE" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{4221CAB4-B4C0-5746-BDF4-C3FC111D5F78}" name="VALUTA" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{530400BE-E6AA-4A47-B046-BF29D0205198}" name="CLASSE" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{99BE53A6-82BE-7C4C-8EDB-FC2585DE7E29}" name="SIMBOLO" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{79CB9D70-57D7-004E-8DD2-11CA0A269F24}" name="DESCRIZIONE" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{4221CAB4-B4C0-5746-BDF4-C3FC111D5F78}" name="VALUTA" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{530400BE-E6AA-4A47-B046-BF29D0205198}" name="CLASSE" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -17319,400 +17393,379 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C714FF38-E71E-3648-9A7A-13401C8B9393}">
-  <dimension ref="A1:N27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="11"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" customWidth="1"/>
-    <col min="2" max="2" width="106.5" customWidth="1"/>
+    <col min="1" max="1" width="11.83203125" style="237" customWidth="1"/>
+    <col min="2" max="2" width="106.5" style="237" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="237"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" s="224" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="235" t="s">
         <v>2120</v>
       </c>
-      <c r="B1" s="225" t="s">
+      <c r="B1" s="236" t="s">
         <v>2121</v>
       </c>
-      <c r="C1" s="221" t="s">
+      <c r="C1" s="237" t="s">
         <v>2122</v>
       </c>
-      <c r="D1" s="221" t="s">
+      <c r="D1" s="237" t="s">
         <v>2703</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="194" t="s">
+    <row r="2" spans="1:4">
+      <c r="A2" s="235" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="240" t="s">
+        <v>2747</v>
+      </c>
+      <c r="C2" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="237" t="s">
+        <v>2748</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="235" t="s">
         <v>2619</v>
       </c>
-      <c r="B2" s="222" t="s">
-        <v>2620</v>
-      </c>
-      <c r="C2" s="196" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="196" t="s">
+      <c r="B3" s="238" t="s">
+        <v>2724</v>
+      </c>
+      <c r="C3" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="237" t="s">
         <v>2696</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
-      <c r="A3" s="196" t="s">
+    <row r="4" spans="1:4">
+      <c r="A4" s="237" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B4" s="238" t="s">
+        <v>2734</v>
+      </c>
+      <c r="C4" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="237" t="s">
+        <v>2635</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="237" t="s">
+        <v>2706</v>
+      </c>
+      <c r="B5" s="238" t="s">
+        <v>2731</v>
+      </c>
+      <c r="C5" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="237" t="s">
+        <v>2708</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="237" t="s">
         <v>2668</v>
       </c>
-      <c r="B3" s="196" t="s">
-        <v>2669</v>
-      </c>
-      <c r="C3" s="196" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="196" t="s">
+      <c r="B6" s="237" t="s">
+        <v>2725</v>
+      </c>
+      <c r="C6" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="237" t="s">
         <v>2673</v>
       </c>
-      <c r="E3" s="48"/>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" s="196" t="s">
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="237" t="s">
         <v>1089</v>
       </c>
-      <c r="B4" s="196" t="s">
-        <v>2674</v>
-      </c>
-      <c r="C4" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="196" t="s">
+      <c r="B7" s="237" t="s">
+        <v>2726</v>
+      </c>
+      <c r="C7" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="237" t="s">
         <v>2680</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="45">
-      <c r="A5" s="223" t="s">
+    <row r="8" spans="1:4">
+      <c r="A8" s="239" t="s">
         <v>2704</v>
       </c>
-      <c r="B5" s="180" t="s">
-        <v>2705</v>
-      </c>
-      <c r="C5" s="196" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="196" t="s">
+      <c r="B8" s="237" t="s">
+        <v>2727</v>
+      </c>
+      <c r="C8" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="237" t="s">
         <v>2685</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
-      <c r="A6" s="196" t="s">
+    <row r="9" spans="1:4">
+      <c r="A9" s="237" t="s">
         <v>2681</v>
       </c>
-      <c r="B6" s="196" t="s">
-        <v>2682</v>
-      </c>
-      <c r="C6" s="196" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="196" t="s">
+      <c r="B9" s="237" t="s">
+        <v>2728</v>
+      </c>
+      <c r="C9" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="237" t="s">
         <v>2686</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="45">
-      <c r="A7" s="196" t="s">
-        <v>2706</v>
-      </c>
-      <c r="B7" s="180" t="s">
-        <v>2707</v>
-      </c>
-      <c r="C7" s="196" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="196" t="s">
-        <v>2708</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="196" t="s">
+    <row r="10" spans="1:4">
+      <c r="A10" s="237" t="s">
         <v>2683</v>
       </c>
-      <c r="B8" s="196" t="s">
-        <v>2684</v>
-      </c>
-      <c r="C8" s="196" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="196" t="s">
+      <c r="B10" s="237" t="s">
+        <v>2729</v>
+      </c>
+      <c r="C10" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="237" t="s">
         <v>2687</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="223" t="s">
+    <row r="11" spans="1:4">
+      <c r="A11" s="239" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="196" t="s">
-        <v>832</v>
-      </c>
-      <c r="C9" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="196" t="s">
+      <c r="B11" s="237" t="s">
+        <v>2730</v>
+      </c>
+      <c r="C11" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="237" t="s">
         <v>2691</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
-      <c r="A10" s="196" t="s">
+    <row r="12" spans="1:4">
+      <c r="A12" s="237" t="s">
+        <v>1872</v>
+      </c>
+      <c r="B12" s="237" t="s">
+        <v>2733</v>
+      </c>
+      <c r="C12" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="237" t="s">
+        <v>2694</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="237" t="s">
         <v>833</v>
       </c>
-      <c r="B10" s="196" t="s">
-        <v>834</v>
-      </c>
-      <c r="C10" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="196" t="s">
+      <c r="B13" s="237" t="s">
+        <v>2732</v>
+      </c>
+      <c r="C13" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="237" t="s">
         <v>2692</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
-      <c r="A11" s="196" t="s">
-        <v>1872</v>
-      </c>
-      <c r="B11" s="196" t="s">
-        <v>2690</v>
-      </c>
-      <c r="C11" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="196" t="s">
-        <v>2694</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12" s="223" t="s">
-        <v>2622</v>
-      </c>
-      <c r="B12" s="196" t="s">
-        <v>2625</v>
-      </c>
-      <c r="C12" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="196" t="s">
-        <v>2634</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
-      <c r="A13" s="196" t="s">
-        <v>1091</v>
-      </c>
-      <c r="B13" s="196" t="s">
-        <v>2629</v>
-      </c>
-      <c r="C13" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="196" t="s">
-        <v>2635</v>
-      </c>
-      <c r="K13" s="48"/>
-      <c r="L13" s="48"/>
-      <c r="M13" s="48"/>
-      <c r="N13" s="48"/>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="A14" s="196" t="s">
+    <row r="14" spans="1:4">
+      <c r="A14" s="237" t="s">
         <v>2636</v>
       </c>
-      <c r="B14" s="196" t="s">
-        <v>2637</v>
-      </c>
-      <c r="C14" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="196" t="s">
+      <c r="B14" s="237" t="s">
+        <v>2735</v>
+      </c>
+      <c r="C14" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="237" t="s">
         <v>2640</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
-      <c r="A15" s="196" t="s">
+    <row r="15" spans="1:4">
+      <c r="A15" s="237" t="s">
         <v>1090</v>
       </c>
-      <c r="B15" s="196" t="s">
-        <v>1316</v>
-      </c>
-      <c r="C15" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="196" t="s">
+      <c r="B15" s="237" t="s">
+        <v>2736</v>
+      </c>
+      <c r="C15" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="237" t="s">
         <v>2644</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
-      <c r="A16" s="223" t="s">
+    <row r="16" spans="1:4">
+      <c r="A16" s="239" t="s">
         <v>2720</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="239" t="s">
+        <v>2737</v>
+      </c>
+      <c r="C16" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="237" t="s">
+        <v>2655</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="239" t="s">
+        <v>2177</v>
+      </c>
+      <c r="B17" s="239" t="s">
+        <v>2738</v>
+      </c>
+      <c r="C17" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="237" t="s">
+        <v>2655</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="239" t="s">
         <v>2721</v>
       </c>
-      <c r="C16" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="196" t="s">
+      <c r="B18" s="239" t="s">
+        <v>2739</v>
+      </c>
+      <c r="C18" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="237" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="223" t="s">
-        <v>2177</v>
-      </c>
-      <c r="B17" s="32" t="s">
+    <row r="19" spans="1:4">
+      <c r="A19" s="237" t="s">
+        <v>2656</v>
+      </c>
+      <c r="B19" s="237" t="s">
+        <v>2740</v>
+      </c>
+      <c r="C19" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="237" t="s">
+        <v>2660</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="237" t="s">
+        <v>2710</v>
+      </c>
+      <c r="B20" s="238" t="s">
+        <v>2741</v>
+      </c>
+      <c r="C20" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="237" t="s">
+        <v>2660</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="237" t="s">
+        <v>2712</v>
+      </c>
+      <c r="B21" s="238" t="s">
+        <v>2742</v>
+      </c>
+      <c r="C21" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="237" t="s">
+        <v>2662</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="239" t="s">
+        <v>2663</v>
+      </c>
+      <c r="B22" s="237" t="s">
+        <v>2743</v>
+      </c>
+      <c r="C22" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="237" t="s">
+        <v>2666</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="239" t="s">
         <v>2722</v>
       </c>
-      <c r="C17" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="196" t="s">
-        <v>2655</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="223" t="s">
-        <v>2723</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>2724</v>
-      </c>
-      <c r="C18" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="196" t="s">
-        <v>2655</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="196" t="s">
-        <v>2656</v>
-      </c>
-      <c r="B19" s="196" t="s">
-        <v>2657</v>
-      </c>
-      <c r="C19" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="196" t="s">
-        <v>2660</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="45">
-      <c r="A20" s="196" t="s">
-        <v>2710</v>
-      </c>
-      <c r="B20" s="180" t="s">
-        <v>2711</v>
-      </c>
-      <c r="C20" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="196" t="s">
-        <v>2660</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="45">
-      <c r="A21" s="196" t="s">
-        <v>2712</v>
-      </c>
-      <c r="B21" s="180" t="s">
-        <v>2713</v>
-      </c>
-      <c r="C21" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="196" t="s">
-        <v>2662</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="45">
-      <c r="A22" s="223" t="s">
-        <v>2714</v>
-      </c>
-      <c r="B22" s="180" t="s">
-        <v>884</v>
-      </c>
-      <c r="C22" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="196" t="s">
-        <v>2662</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="223" t="s">
-        <v>2663</v>
-      </c>
-      <c r="B23" s="196" t="s">
-        <v>2664</v>
-      </c>
-      <c r="C23" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="196" t="s">
+      <c r="B23" s="239" t="s">
+        <v>2744</v>
+      </c>
+      <c r="C23" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="237" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="32" t="s">
-        <v>2725</v>
-      </c>
-      <c r="B24" s="32" t="s">
-        <v>2726</v>
-      </c>
-      <c r="C24" s="196"/>
-      <c r="D24" s="196"/>
-    </row>
-    <row r="25" spans="1:4" ht="45">
-      <c r="A25" s="196" t="s">
+      <c r="A24" s="237" t="s">
         <v>2718</v>
       </c>
-      <c r="B25" s="180" t="s">
-        <v>2727</v>
-      </c>
-      <c r="C25" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="196" t="s">
+      <c r="B24" s="238" t="s">
+        <v>2745</v>
+      </c>
+      <c r="C24" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="237" t="s">
         <v>2667</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="196" t="s">
+    <row r="25" spans="1:4">
+      <c r="A25" s="237" t="s">
         <v>2697</v>
       </c>
-      <c r="B26" s="196" t="s">
-        <v>2698</v>
-      </c>
-      <c r="C26" s="196" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="196" t="s">
+      <c r="B25" s="237" t="s">
+        <v>2746</v>
+      </c>
+      <c r="C25" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="237" t="s">
         <v>2089</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="196"/>
-      <c r="B27" s="196"/>
-      <c r="C27" s="196"/>
-      <c r="D27" s="196"/>
     </row>
   </sheetData>
   <phoneticPr fontId="95" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A23" r:id="rId1" display="http://xgin.de/" xr:uid="{6D042F4B-B1B6-714D-834A-FF03BB9AF65F}"/>
-    <hyperlink ref="A12" r:id="rId2" display="http://iusq.de/" xr:uid="{B40808EF-D56C-CF4A-8448-3B54D7C1E5D4}"/>
-    <hyperlink ref="A9" r:id="rId3" display="http://zprv.de/" xr:uid="{AE8F80AC-32A6-C643-BEE6-694ECBB145F6}"/>
-    <hyperlink ref="A5" r:id="rId4" display="http://iusg.de/" xr:uid="{C28C7857-119A-4744-B0BB-4DDEA3E95E35}"/>
-    <hyperlink ref="B16" r:id="rId5" display="https://finance.yahoo.com/quote/CSBGE3.MI/" xr:uid="{07F4F9CA-E0FA-1C49-87F4-4EBCF7177C7D}"/>
-    <hyperlink ref="B17" r:id="rId6" display="https://finance.yahoo.com/quote/CSBGE7.MI/" xr:uid="{02FC7EA0-25C6-E34E-AB6A-3622B551A50D}"/>
-    <hyperlink ref="B18" r:id="rId7" display="https://finance.yahoo.com/quote/SXRQ.DE/" xr:uid="{4E4D2C26-5E71-C644-AF09-EF7691622628}"/>
-    <hyperlink ref="A24" r:id="rId8" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{6DA783E3-A09C-7C47-88D8-23C14B21E7FE}"/>
-    <hyperlink ref="B24" r:id="rId9" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{894A731F-3358-3D4B-A900-50AD652ED5AE}"/>
+    <hyperlink ref="A22" r:id="rId1" display="http://xgin.de/" xr:uid="{6D042F4B-B1B6-714D-834A-FF03BB9AF65F}"/>
+    <hyperlink ref="A11" r:id="rId2" display="http://zprv.de/" xr:uid="{AE8F80AC-32A6-C643-BEE6-694ECBB145F6}"/>
+    <hyperlink ref="A8" r:id="rId3" display="http://iusg.de/" xr:uid="{C28C7857-119A-4744-B0BB-4DDEA3E95E35}"/>
+    <hyperlink ref="B16" r:id="rId4" display="https://finance.yahoo.com/quote/CSBGE3.MI/" xr:uid="{07F4F9CA-E0FA-1C49-87F4-4EBCF7177C7D}"/>
+    <hyperlink ref="B17" r:id="rId5" display="https://finance.yahoo.com/quote/CSBGE7.MI/" xr:uid="{02FC7EA0-25C6-E34E-AB6A-3622B551A50D}"/>
+    <hyperlink ref="B18" r:id="rId6" display="https://finance.yahoo.com/quote/SXRQ.DE/" xr:uid="{4E4D2C26-5E71-C644-AF09-EF7691622628}"/>
+    <hyperlink ref="A23" r:id="rId7" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{6DA783E3-A09C-7C47-88D8-23C14B21E7FE}"/>
+    <hyperlink ref="B23" r:id="rId8" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{894A731F-3358-3D4B-A900-50AD652ED5AE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId10"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
@@ -17728,20 +17781,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17">
-      <c r="A1" s="228" t="s">
+      <c r="A1" s="233" t="s">
         <v>2346</v>
       </c>
-      <c r="B1" s="227"/>
-      <c r="C1" s="227"/>
-      <c r="D1" s="227"/>
+      <c r="B1" s="232"/>
+      <c r="C1" s="232"/>
+      <c r="D1" s="232"/>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="229" t="s">
+      <c r="A2" s="234" t="s">
         <v>2347</v>
       </c>
-      <c r="B2" s="227"/>
-      <c r="C2" s="227"/>
-      <c r="D2" s="227"/>
+      <c r="B2" s="232"/>
+      <c r="C2" s="232"/>
+      <c r="D2" s="232"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="181" t="s">
@@ -17758,12 +17811,12 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="226" t="s">
+      <c r="A4" s="231" t="s">
         <v>2349</v>
       </c>
-      <c r="B4" s="227"/>
-      <c r="C4" s="227"/>
-      <c r="D4" s="227"/>
+      <c r="B4" s="232"/>
+      <c r="C4" s="232"/>
+      <c r="D4" s="232"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="182" t="s">
@@ -17990,12 +18043,12 @@
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="226" t="s">
+      <c r="A21" s="231" t="s">
         <v>2377</v>
       </c>
-      <c r="B21" s="227"/>
-      <c r="C21" s="227"/>
-      <c r="D21" s="227"/>
+      <c r="B21" s="232"/>
+      <c r="C21" s="232"/>
+      <c r="D21" s="232"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="186" t="s">
@@ -18040,12 +18093,12 @@
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="226" t="s">
+      <c r="A25" s="231" t="s">
         <v>2384</v>
       </c>
-      <c r="B25" s="227"/>
-      <c r="C25" s="227"/>
-      <c r="D25" s="227"/>
+      <c r="B25" s="232"/>
+      <c r="C25" s="232"/>
+      <c r="D25" s="232"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="186" t="s">
@@ -18090,12 +18143,12 @@
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="226" t="s">
+      <c r="A29" s="231" t="s">
         <v>2391</v>
       </c>
-      <c r="B29" s="227"/>
-      <c r="C29" s="227"/>
-      <c r="D29" s="227"/>
+      <c r="B29" s="232"/>
+      <c r="C29" s="232"/>
+      <c r="D29" s="232"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="186" t="s">
@@ -18140,12 +18193,12 @@
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="226" t="s">
+      <c r="A33" s="231" t="s">
         <v>2395</v>
       </c>
-      <c r="B33" s="227"/>
-      <c r="C33" s="227"/>
-      <c r="D33" s="227"/>
+      <c r="B33" s="232"/>
+      <c r="C33" s="232"/>
+      <c r="D33" s="232"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="186" t="s">
@@ -18204,12 +18257,12 @@
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="226" t="s">
+      <c r="A38" s="231" t="s">
         <v>2403</v>
       </c>
-      <c r="B38" s="227"/>
-      <c r="C38" s="227"/>
-      <c r="D38" s="227"/>
+      <c r="B38" s="232"/>
+      <c r="C38" s="232"/>
+      <c r="D38" s="232"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="190" t="s">
@@ -18254,12 +18307,12 @@
       </c>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="226" t="s">
+      <c r="A42" s="231" t="s">
         <v>2410</v>
       </c>
-      <c r="B42" s="227"/>
-      <c r="C42" s="227"/>
-      <c r="D42" s="227"/>
+      <c r="B42" s="232"/>
+      <c r="C42" s="232"/>
+      <c r="D42" s="232"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="190" t="s">
@@ -18304,12 +18357,12 @@
       </c>
     </row>
     <row r="46" spans="1:4">
-      <c r="A46" s="226" t="s">
+      <c r="A46" s="231" t="s">
         <v>2417</v>
       </c>
-      <c r="B46" s="227"/>
-      <c r="C46" s="227"/>
-      <c r="D46" s="227"/>
+      <c r="B46" s="232"/>
+      <c r="C46" s="232"/>
+      <c r="D46" s="232"/>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="190" t="s">
@@ -18354,12 +18407,12 @@
       </c>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="226" t="s">
+      <c r="A50" s="231" t="s">
         <v>2424</v>
       </c>
-      <c r="B50" s="227"/>
-      <c r="C50" s="227"/>
-      <c r="D50" s="227"/>
+      <c r="B50" s="232"/>
+      <c r="C50" s="232"/>
+      <c r="D50" s="232"/>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="190" t="s">
@@ -18404,12 +18457,12 @@
       </c>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" s="226" t="s">
+      <c r="A54" s="231" t="s">
         <v>2431</v>
       </c>
-      <c r="B54" s="227"/>
-      <c r="C54" s="227"/>
-      <c r="D54" s="227"/>
+      <c r="B54" s="232"/>
+      <c r="C54" s="232"/>
+      <c r="D54" s="232"/>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="190" t="s">
@@ -18454,12 +18507,12 @@
       </c>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" s="226" t="s">
+      <c r="A58" s="231" t="s">
         <v>2437</v>
       </c>
-      <c r="B58" s="227"/>
-      <c r="C58" s="227"/>
-      <c r="D58" s="227"/>
+      <c r="B58" s="232"/>
+      <c r="C58" s="232"/>
+      <c r="D58" s="232"/>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="190" t="s">
@@ -18504,12 +18557,12 @@
       </c>
     </row>
     <row r="62" spans="1:4">
-      <c r="A62" s="226" t="s">
+      <c r="A62" s="231" t="s">
         <v>2444</v>
       </c>
-      <c r="B62" s="227"/>
-      <c r="C62" s="227"/>
-      <c r="D62" s="227"/>
+      <c r="B62" s="232"/>
+      <c r="C62" s="232"/>
+      <c r="D62" s="232"/>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="190" t="s">
@@ -18540,12 +18593,12 @@
       </c>
     </row>
     <row r="65" spans="1:4">
-      <c r="A65" s="226" t="s">
+      <c r="A65" s="231" t="s">
         <v>2449</v>
       </c>
-      <c r="B65" s="227"/>
-      <c r="C65" s="227"/>
-      <c r="D65" s="227"/>
+      <c r="B65" s="232"/>
+      <c r="C65" s="232"/>
+      <c r="D65" s="232"/>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="186" t="s">
@@ -18590,12 +18643,12 @@
       </c>
     </row>
     <row r="69" spans="1:4">
-      <c r="A69" s="226" t="s">
+      <c r="A69" s="231" t="s">
         <v>2455</v>
       </c>
-      <c r="B69" s="227"/>
-      <c r="C69" s="227"/>
-      <c r="D69" s="227"/>
+      <c r="B69" s="232"/>
+      <c r="C69" s="232"/>
+      <c r="D69" s="232"/>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="186" t="s">
@@ -18626,12 +18679,12 @@
       </c>
     </row>
     <row r="72" spans="1:4">
-      <c r="A72" s="226" t="s">
+      <c r="A72" s="231" t="s">
         <v>2460</v>
       </c>
-      <c r="B72" s="227"/>
-      <c r="C72" s="227"/>
-      <c r="D72" s="227"/>
+      <c r="B72" s="232"/>
+      <c r="C72" s="232"/>
+      <c r="D72" s="232"/>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="190" t="s">
@@ -18676,12 +18729,12 @@
       </c>
     </row>
     <row r="76" spans="1:4">
-      <c r="A76" s="226" t="s">
+      <c r="A76" s="231" t="s">
         <v>2467</v>
       </c>
-      <c r="B76" s="227"/>
-      <c r="C76" s="227"/>
-      <c r="D76" s="227"/>
+      <c r="B76" s="232"/>
+      <c r="C76" s="232"/>
+      <c r="D76" s="232"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="190" t="s">
@@ -18726,12 +18779,12 @@
       </c>
     </row>
     <row r="80" spans="1:4">
-      <c r="A80" s="226" t="s">
+      <c r="A80" s="231" t="s">
         <v>2474</v>
       </c>
-      <c r="B80" s="227"/>
-      <c r="C80" s="227"/>
-      <c r="D80" s="227"/>
+      <c r="B80" s="232"/>
+      <c r="C80" s="232"/>
+      <c r="D80" s="232"/>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="190" t="s">
@@ -18777,6 +18830,13 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A76:D76"/>
     <mergeCell ref="A54:D54"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -18789,13 +18849,6 @@
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A46:D46"/>
     <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A76:D76"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -22907,812 +22960,812 @@
   <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" style="233" customWidth="1"/>
-    <col min="2" max="2" width="78.83203125" style="233" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="233"/>
+    <col min="1" max="1" width="11.83203125" style="224" customWidth="1"/>
+    <col min="2" max="2" width="78.83203125" style="224" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="224"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="234" t="s">
+      <c r="A1" s="225" t="s">
         <v>2120</v>
       </c>
-      <c r="B1" s="237" t="s">
+      <c r="B1" s="228" t="s">
         <v>2121</v>
       </c>
-      <c r="C1" s="233" t="s">
+      <c r="C1" s="224" t="s">
         <v>2122</v>
       </c>
-      <c r="D1" s="233" t="s">
+      <c r="D1" s="224" t="s">
         <v>2703</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="230" t="s">
+      <c r="A2" s="221" t="s">
         <v>820</v>
       </c>
-      <c r="B2" s="231" t="s">
+      <c r="B2" s="222" t="s">
         <v>1032</v>
       </c>
-      <c r="C2" s="232" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="233" t="s">
+      <c r="C2" s="223" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="224" t="s">
         <v>2695</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="234" t="s">
+      <c r="A3" s="225" t="s">
         <v>2619</v>
       </c>
-      <c r="B3" s="231" t="s">
+      <c r="B3" s="222" t="s">
         <v>2620</v>
       </c>
-      <c r="C3" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="233" t="s">
+      <c r="C3" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="224" t="s">
         <v>2696</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="233" t="s">
+      <c r="A4" s="224" t="s">
         <v>2668</v>
       </c>
-      <c r="B4" s="233" t="s">
+      <c r="B4" s="224" t="s">
         <v>2669</v>
       </c>
-      <c r="C4" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="233" t="s">
+      <c r="C4" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="224" t="s">
         <v>2673</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="235" t="s">
+      <c r="A5" s="226" t="s">
         <v>2670</v>
       </c>
-      <c r="B5" s="233" t="s">
+      <c r="B5" s="224" t="s">
         <v>2671</v>
       </c>
-      <c r="C5" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="233" t="s">
+      <c r="C5" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="224" t="s">
         <v>2673</v>
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="233" t="s">
+      <c r="A6" s="224" t="s">
         <v>2132</v>
       </c>
-      <c r="B6" s="233" t="s">
+      <c r="B6" s="224" t="s">
         <v>2672</v>
       </c>
-      <c r="C6" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="233" t="s">
+      <c r="C6" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="224" t="s">
         <v>2673</v>
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="233" t="s">
+      <c r="A7" s="224" t="s">
         <v>1089</v>
       </c>
-      <c r="B7" s="233" t="s">
+      <c r="B7" s="224" t="s">
         <v>2674</v>
       </c>
-      <c r="C7" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="233" t="s">
+      <c r="C7" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="224" t="s">
         <v>2680</v>
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="235" t="s">
+      <c r="A8" s="226" t="s">
         <v>2675</v>
       </c>
-      <c r="B8" s="233" t="s">
+      <c r="B8" s="224" t="s">
         <v>2676</v>
       </c>
-      <c r="C8" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="233" t="s">
+      <c r="C8" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="224" t="s">
         <v>2680</v>
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="233" t="s">
+      <c r="A9" s="224" t="s">
         <v>2677</v>
       </c>
-      <c r="B9" s="233" t="s">
+      <c r="B9" s="224" t="s">
         <v>2678</v>
       </c>
-      <c r="C9" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="233" t="s">
+      <c r="C9" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="224" t="s">
         <v>2680</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="233" t="s">
+      <c r="A10" s="224" t="s">
         <v>2679</v>
       </c>
-      <c r="B10" s="233" t="s">
+      <c r="B10" s="224" t="s">
         <v>2678</v>
       </c>
-      <c r="C10" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="233" t="s">
+      <c r="C10" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="224" t="s">
         <v>2680</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="235" t="s">
+      <c r="A11" s="226" t="s">
         <v>2704</v>
       </c>
-      <c r="B11" s="231" t="s">
+      <c r="B11" s="222" t="s">
         <v>2705</v>
       </c>
-      <c r="C11" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="233" t="s">
+      <c r="C11" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="224" t="s">
         <v>2685</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="233" t="s">
+      <c r="A12" s="224" t="s">
         <v>2681</v>
       </c>
-      <c r="B12" s="233" t="s">
+      <c r="B12" s="224" t="s">
         <v>2682</v>
       </c>
-      <c r="C12" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="233" t="s">
+      <c r="C12" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="224" t="s">
         <v>2686</v>
       </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="233" t="s">
+      <c r="A13" s="224" t="s">
         <v>2706</v>
       </c>
-      <c r="B13" s="231" t="s">
+      <c r="B13" s="222" t="s">
         <v>2707</v>
       </c>
-      <c r="C13" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="233" t="s">
+      <c r="C13" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="224" t="s">
         <v>2708</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="233" t="s">
+      <c r="A14" s="224" t="s">
         <v>2683</v>
       </c>
-      <c r="B14" s="233" t="s">
+      <c r="B14" s="224" t="s">
         <v>2684</v>
       </c>
-      <c r="C14" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="233" t="s">
+      <c r="C14" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="224" t="s">
         <v>2687</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="235" t="s">
+      <c r="A15" s="226" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="233" t="s">
+      <c r="B15" s="224" t="s">
         <v>832</v>
       </c>
-      <c r="C15" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="233" t="s">
+      <c r="C15" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="224" t="s">
         <v>2691</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="233" t="s">
+      <c r="A16" s="224" t="s">
         <v>833</v>
       </c>
-      <c r="B16" s="233" t="s">
+      <c r="B16" s="224" t="s">
         <v>834</v>
       </c>
-      <c r="C16" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="233" t="s">
+      <c r="C16" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="224" t="s">
         <v>2692</v>
       </c>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="233" t="s">
+      <c r="A17" s="224" t="s">
         <v>2688</v>
       </c>
-      <c r="B17" s="233" t="s">
+      <c r="B17" s="224" t="s">
         <v>2689</v>
       </c>
-      <c r="C17" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="233" t="s">
+      <c r="C17" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="224" t="s">
         <v>2693</v>
       </c>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" s="233" t="s">
+      <c r="A18" s="224" t="s">
         <v>1872</v>
       </c>
-      <c r="B18" s="233" t="s">
+      <c r="B18" s="224" t="s">
         <v>2690</v>
       </c>
-      <c r="C18" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="233" t="s">
+      <c r="C18" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="224" t="s">
         <v>2694</v>
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="233" t="s">
+      <c r="A19" s="224" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="233" t="s">
+      <c r="B19" s="224" t="s">
         <v>2621</v>
       </c>
-      <c r="C19" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="233" t="s">
+      <c r="C19" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="224" t="s">
         <v>2634</v>
       </c>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" s="235" t="s">
+      <c r="A20" s="226" t="s">
         <v>2622</v>
       </c>
-      <c r="B20" s="233" t="s">
+      <c r="B20" s="224" t="s">
         <v>2625</v>
       </c>
-      <c r="C20" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="233" t="s">
+      <c r="C20" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="224" t="s">
         <v>2634</v>
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="233" t="s">
+      <c r="A21" s="224" t="s">
         <v>2623</v>
       </c>
-      <c r="B21" s="233" t="s">
+      <c r="B21" s="224" t="s">
         <v>2626</v>
       </c>
-      <c r="C21" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="233" t="s">
+      <c r="C21" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="224" t="s">
         <v>2634</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="235" t="s">
+      <c r="A22" s="226" t="s">
         <v>1126</v>
       </c>
-      <c r="B22" s="233" t="s">
+      <c r="B22" s="224" t="s">
         <v>2627</v>
       </c>
-      <c r="C22" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="233" t="s">
+      <c r="C22" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="224" t="s">
         <v>2634</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="233" t="s">
+      <c r="A23" s="224" t="s">
         <v>2624</v>
       </c>
-      <c r="B23" s="233" t="s">
+      <c r="B23" s="224" t="s">
         <v>2628</v>
       </c>
-      <c r="C23" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="233" t="s">
+      <c r="C23" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="224" t="s">
         <v>2634</v>
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="233" t="s">
+      <c r="A24" s="224" t="s">
         <v>1091</v>
       </c>
-      <c r="B24" s="233" t="s">
+      <c r="B24" s="224" t="s">
         <v>2629</v>
       </c>
-      <c r="C24" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D24" s="233" t="s">
+      <c r="C24" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="224" t="s">
         <v>2635</v>
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="235" t="s">
+      <c r="A25" s="226" t="s">
         <v>2630</v>
       </c>
-      <c r="B25" s="233" t="s">
+      <c r="B25" s="224" t="s">
         <v>2631</v>
       </c>
-      <c r="C25" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="233" t="s">
+      <c r="C25" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="224" t="s">
         <v>2635</v>
       </c>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" s="233" t="s">
+      <c r="A26" s="224" t="s">
         <v>2632</v>
       </c>
-      <c r="B26" s="233" t="s">
+      <c r="B26" s="224" t="s">
         <v>2633</v>
       </c>
-      <c r="C26" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="233" t="s">
+      <c r="C26" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="224" t="s">
         <v>2635</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="233" t="s">
+      <c r="A27" s="224" t="s">
         <v>1753</v>
       </c>
-      <c r="B27" s="233" t="s">
+      <c r="B27" s="224" t="s">
         <v>831</v>
       </c>
-      <c r="C27" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D27" s="233" t="s">
+      <c r="C27" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" s="224" t="s">
         <v>2635</v>
       </c>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" s="233" t="s">
+      <c r="A28" s="224" t="s">
         <v>2636</v>
       </c>
-      <c r="B28" s="233" t="s">
+      <c r="B28" s="224" t="s">
         <v>2637</v>
       </c>
-      <c r="C28" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D28" s="233" t="s">
+      <c r="C28" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="224" t="s">
         <v>2640</v>
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="235" t="s">
+      <c r="A29" s="226" t="s">
         <v>2638</v>
       </c>
-      <c r="B29" s="233" t="s">
+      <c r="B29" s="224" t="s">
         <v>2639</v>
       </c>
-      <c r="C29" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D29" s="233" t="s">
+      <c r="C29" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="224" t="s">
         <v>2640</v>
       </c>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" s="233" t="s">
+      <c r="A30" s="224" t="s">
         <v>1090</v>
       </c>
-      <c r="B30" s="233" t="s">
+      <c r="B30" s="224" t="s">
         <v>1316</v>
       </c>
-      <c r="C30" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D30" s="233" t="s">
+      <c r="C30" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" s="224" t="s">
         <v>2644</v>
       </c>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="233" t="s">
+      <c r="A31" s="224" t="s">
         <v>2324</v>
       </c>
-      <c r="B31" s="233" t="s">
+      <c r="B31" s="224" t="s">
         <v>2641</v>
       </c>
-      <c r="C31" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D31" s="233" t="s">
+      <c r="C31" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" s="224" t="s">
         <v>2644</v>
       </c>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="233" t="s">
+      <c r="A32" s="224" t="s">
         <v>2642</v>
       </c>
-      <c r="B32" s="233" t="s">
+      <c r="B32" s="224" t="s">
         <v>2643</v>
       </c>
-      <c r="C32" s="233" t="s">
-        <v>29</v>
-      </c>
-      <c r="D32" s="233" t="s">
+      <c r="C32" s="224" t="s">
+        <v>29</v>
+      </c>
+      <c r="D32" s="224" t="s">
         <v>2644</v>
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="233" t="s">
+      <c r="A33" s="224" t="s">
         <v>2645</v>
       </c>
-      <c r="B33" s="233" t="s">
+      <c r="B33" s="224" t="s">
         <v>2646</v>
       </c>
-      <c r="C33" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D33" s="233" t="s">
+      <c r="C33" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D33" s="224" t="s">
         <v>2651</v>
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="233" t="s">
+      <c r="A34" s="224" t="s">
         <v>2647</v>
       </c>
-      <c r="B34" s="233" t="s">
+      <c r="B34" s="224" t="s">
         <v>2648</v>
       </c>
-      <c r="C34" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D34" s="233" t="s">
+      <c r="C34" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" s="224" t="s">
         <v>2651</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="235" t="s">
+      <c r="A35" s="226" t="s">
         <v>2649</v>
       </c>
-      <c r="B35" s="233" t="s">
+      <c r="B35" s="224" t="s">
         <v>2650</v>
       </c>
-      <c r="C35" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D35" s="233" t="s">
+      <c r="C35" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D35" s="224" t="s">
         <v>2655</v>
       </c>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" s="235" t="s">
+      <c r="A36" s="226" t="s">
         <v>2709</v>
       </c>
-      <c r="B36" s="233" t="s">
+      <c r="B36" s="224" t="s">
         <v>2652</v>
       </c>
-      <c r="C36" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D36" s="233" t="s">
+      <c r="C36" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D36" s="224" t="s">
         <v>2655</v>
       </c>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="235" t="s">
+      <c r="A37" s="226" t="s">
         <v>2097</v>
       </c>
-      <c r="B37" s="233" t="s">
+      <c r="B37" s="224" t="s">
         <v>2653</v>
       </c>
-      <c r="C37" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D37" s="233" t="s">
+      <c r="C37" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D37" s="224" t="s">
         <v>2655</v>
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="235" t="s">
+      <c r="A38" s="226" t="s">
         <v>1100</v>
       </c>
-      <c r="B38" s="233" t="s">
+      <c r="B38" s="224" t="s">
         <v>2654</v>
       </c>
-      <c r="C38" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D38" s="233" t="s">
+      <c r="C38" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D38" s="224" t="s">
         <v>2655</v>
       </c>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="233" t="s">
+      <c r="A39" s="224" t="s">
         <v>2656</v>
       </c>
-      <c r="B39" s="233" t="s">
+      <c r="B39" s="224" t="s">
         <v>2657</v>
       </c>
-      <c r="C39" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D39" s="233" t="s">
+      <c r="C39" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D39" s="224" t="s">
         <v>2660</v>
       </c>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="233" t="s">
+      <c r="A40" s="224" t="s">
         <v>2710</v>
       </c>
-      <c r="B40" s="231" t="s">
+      <c r="B40" s="222" t="s">
         <v>2711</v>
       </c>
-      <c r="C40" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D40" s="233" t="s">
+      <c r="C40" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" s="224" t="s">
         <v>2660</v>
       </c>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="235" t="s">
+      <c r="A41" s="226" t="s">
         <v>2658</v>
       </c>
-      <c r="B41" s="233" t="s">
+      <c r="B41" s="224" t="s">
         <v>2659</v>
       </c>
-      <c r="C41" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D41" s="233" t="s">
+      <c r="C41" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D41" s="224" t="s">
         <v>2660</v>
       </c>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="235" t="s">
+      <c r="A42" s="226" t="s">
         <v>1113</v>
       </c>
-      <c r="B42" s="233" t="s">
+      <c r="B42" s="224" t="s">
         <v>2661</v>
       </c>
-      <c r="C42" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D42" s="233" t="s">
+      <c r="C42" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D42" s="224" t="s">
         <v>2662</v>
       </c>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="233" t="s">
+      <c r="A43" s="224" t="s">
         <v>2712</v>
       </c>
-      <c r="B43" s="231" t="s">
+      <c r="B43" s="222" t="s">
         <v>2713</v>
       </c>
-      <c r="C43" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D43" s="233" t="s">
+      <c r="C43" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D43" s="224" t="s">
         <v>2662</v>
       </c>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" s="235" t="s">
+      <c r="A44" s="226" t="s">
         <v>2714</v>
       </c>
-      <c r="B44" s="231" t="s">
+      <c r="B44" s="222" t="s">
         <v>884</v>
       </c>
-      <c r="C44" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D44" s="233" t="s">
+      <c r="C44" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D44" s="224" t="s">
         <v>2662</v>
       </c>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" s="233" t="s">
+      <c r="A45" s="224" t="s">
         <v>2090</v>
       </c>
-      <c r="B45" s="231" t="s">
+      <c r="B45" s="222" t="s">
         <v>2715</v>
       </c>
-      <c r="C45" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D45" s="233" t="s">
+      <c r="C45" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D45" s="224" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="46" spans="1:4">
-      <c r="A46" s="235" t="s">
+      <c r="A46" s="226" t="s">
         <v>2663</v>
       </c>
-      <c r="B46" s="233" t="s">
+      <c r="B46" s="224" t="s">
         <v>2664</v>
       </c>
-      <c r="C46" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D46" s="233" t="s">
+      <c r="C46" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D46" s="224" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="47" spans="1:4">
-      <c r="A47" s="233" t="s">
+      <c r="A47" s="224" t="s">
         <v>2411</v>
       </c>
-      <c r="B47" s="233" t="s">
+      <c r="B47" s="224" t="s">
         <v>2665</v>
       </c>
-      <c r="C47" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D47" s="233" t="s">
+      <c r="C47" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D47" s="224" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="48" spans="1:4">
-      <c r="A48" s="233" t="s">
+      <c r="A48" s="224" t="s">
         <v>2716</v>
       </c>
-      <c r="B48" s="231" t="s">
+      <c r="B48" s="222" t="s">
         <v>2717</v>
       </c>
-      <c r="C48" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D48" s="233" t="s">
+      <c r="C48" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D48" s="224" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="49" spans="1:9">
-      <c r="A49" s="233" t="s">
+      <c r="A49" s="224" t="s">
         <v>2718</v>
       </c>
-      <c r="B49" s="231" t="s">
+      <c r="B49" s="222" t="s">
         <v>2719</v>
       </c>
-      <c r="C49" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D49" s="233" t="s">
+      <c r="C49" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D49" s="224" t="s">
         <v>2667</v>
       </c>
     </row>
     <row r="50" spans="1:9">
-      <c r="A50" s="233" t="s">
+      <c r="A50" s="224" t="s">
         <v>2697</v>
       </c>
-      <c r="B50" s="233" t="s">
+      <c r="B50" s="224" t="s">
         <v>2698</v>
       </c>
-      <c r="C50" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D50" s="233" t="s">
+      <c r="C50" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D50" s="224" t="s">
         <v>2089</v>
       </c>
     </row>
     <row r="51" spans="1:9">
-      <c r="A51" s="233" t="s">
+      <c r="A51" s="224" t="s">
         <v>2135</v>
       </c>
-      <c r="B51" s="233" t="s">
+      <c r="B51" s="224" t="s">
         <v>1962</v>
       </c>
-      <c r="C51" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D51" s="233" t="s">
+      <c r="C51" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D51" s="224" t="s">
         <v>2089</v>
       </c>
     </row>
     <row r="52" spans="1:9">
-      <c r="A52" s="235" t="s">
+      <c r="A52" s="226" t="s">
         <v>2699</v>
       </c>
-      <c r="B52" s="233" t="s">
+      <c r="B52" s="224" t="s">
         <v>2700</v>
       </c>
-      <c r="C52" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D52" s="233" t="s">
+      <c r="C52" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D52" s="224" t="s">
         <v>2089</v>
       </c>
     </row>
     <row r="53" spans="1:9">
-      <c r="A53" s="233" t="s">
+      <c r="A53" s="224" t="s">
         <v>2701</v>
       </c>
-      <c r="B53" s="233" t="s">
+      <c r="B53" s="224" t="s">
         <v>2702</v>
       </c>
-      <c r="C53" s="233" t="s">
-        <v>28</v>
-      </c>
-      <c r="D53" s="233" t="s">
+      <c r="C53" s="224" t="s">
+        <v>28</v>
+      </c>
+      <c r="D53" s="224" t="s">
         <v>2089</v>
       </c>
     </row>
     <row r="54" spans="1:9">
-      <c r="A54" s="231" t="s">
+      <c r="A54" s="222" t="s">
         <v>2571</v>
       </c>
-      <c r="B54" s="231" t="s">
+      <c r="B54" s="222" t="s">
         <v>2572</v>
       </c>
-      <c r="C54" s="238" t="s">
-        <v>28</v>
-      </c>
-      <c r="D54" s="236" t="s">
-        <v>2728</v>
-      </c>
-      <c r="I54" s="236"/>
+      <c r="C54" s="229" t="s">
+        <v>28</v>
+      </c>
+      <c r="D54" s="227" t="s">
+        <v>2723</v>
+      </c>
+      <c r="I54" s="227"/>
     </row>
     <row r="55" spans="1:9">
-      <c r="A55" s="233" t="s">
+      <c r="A55" s="224" t="s">
         <v>2255</v>
       </c>
-      <c r="B55" s="231" t="s">
+      <c r="B55" s="222" t="s">
         <v>2614</v>
       </c>
-      <c r="C55" s="239" t="s">
-        <v>28</v>
-      </c>
-      <c r="D55" s="236" t="s">
-        <v>2728</v>
-      </c>
-      <c r="I55" s="236"/>
+      <c r="C55" s="230" t="s">
+        <v>28</v>
+      </c>
+      <c r="D55" s="227" t="s">
+        <v>2723</v>
+      </c>
+      <c r="I55" s="227"/>
     </row>
     <row r="56" spans="1:9">
-      <c r="A56" s="233" t="s">
+      <c r="A56" s="224" t="s">
         <v>2615</v>
       </c>
-      <c r="B56" s="231" t="s">
+      <c r="B56" s="222" t="s">
         <v>2616</v>
       </c>
-      <c r="C56" s="239" t="s">
-        <v>28</v>
-      </c>
-      <c r="D56" s="236" t="s">
-        <v>2728</v>
-      </c>
-      <c r="I56" s="236"/>
+      <c r="C56" s="230" t="s">
+        <v>28</v>
+      </c>
+      <c r="D56" s="227" t="s">
+        <v>2723</v>
+      </c>
+      <c r="I56" s="227"/>
     </row>
     <row r="57" spans="1:9">
-      <c r="A57" s="233" t="s">
+      <c r="A57" s="224" t="s">
         <v>2617</v>
       </c>
-      <c r="B57" s="231" t="s">
+      <c r="B57" s="222" t="s">
         <v>2618</v>
       </c>
-      <c r="C57" s="239" t="s">
-        <v>28</v>
-      </c>
-      <c r="D57" s="236" t="s">
-        <v>2728</v>
-      </c>
-      <c r="I57" s="236"/>
+      <c r="C57" s="230" t="s">
+        <v>28</v>
+      </c>
+      <c r="D57" s="227" t="s">
+        <v>2723</v>
+      </c>
+      <c r="I57" s="227"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Aggiunge callback per pulsanti deselect/reset colonne
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TARBIUTH.xlsx
+++ b/TARBIUTH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookpro/Downloads/andcappe_zip/Dashboard/SITO_WEB/Sito personale/portafoglio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76750A06-1780-A740-A3CE-CB2DF706D97E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9173B583-2356-BF4D-A639-A3BD8687E0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4380" yWindow="20" windowWidth="24420" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7566" uniqueCount="2749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7570" uniqueCount="2751">
   <si>
     <t>Simbolo</t>
   </si>
@@ -8558,6 +8558,12 @@
   </si>
   <si>
     <t>Azionario ACWI Vanguard</t>
+  </si>
+  <si>
+    <t>AZ. USA Info Tech SP500</t>
+  </si>
+  <si>
+    <t>Azionari Tech Sp500</t>
   </si>
 </sst>
 </file>
@@ -16263,8 +16269,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D25" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:D25" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D26" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:D26" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{12AF85F4-CF3E-1A44-9197-52CD700ECF69}" name="SIMBOLO" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{D2DEAFE7-7181-F841-96D9-E16F6CD58118}" name="DESCRIZIONE" dataDxfId="4"/>
@@ -17393,7 +17399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C714FF38-E71E-3648-9A7A-13401C8B9393}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="11"/>
   <cols>
     <col min="1" max="1" width="11.83203125" style="237" customWidth="1"/>
@@ -17471,166 +17477,166 @@
         <v>2708</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" ht="15">
       <c r="A6" s="237" t="s">
-        <v>2668</v>
+        <v>59</v>
       </c>
       <c r="B6" s="237" t="s">
-        <v>2725</v>
+        <v>2749</v>
       </c>
       <c r="C6" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="237" t="s">
-        <v>2673</v>
+        <v>28</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>2750</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="237" t="s">
+        <v>2668</v>
+      </c>
+      <c r="B7" s="237" t="s">
+        <v>2725</v>
+      </c>
+      <c r="C7" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="237" t="s">
+        <v>2673</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="237" t="s">
         <v>1089</v>
       </c>
-      <c r="B7" s="237" t="s">
+      <c r="B8" s="237" t="s">
         <v>2726</v>
       </c>
-      <c r="C7" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="237" t="s">
+      <c r="C8" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="237" t="s">
         <v>2680</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="239" t="s">
+    <row r="9" spans="1:4">
+      <c r="A9" s="239" t="s">
         <v>2704</v>
       </c>
-      <c r="B8" s="237" t="s">
+      <c r="B9" s="237" t="s">
         <v>2727</v>
       </c>
-      <c r="C8" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="237" t="s">
+      <c r="C9" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="237" t="s">
         <v>2685</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="237" t="s">
-        <v>2681</v>
-      </c>
-      <c r="B9" s="237" t="s">
-        <v>2728</v>
-      </c>
-      <c r="C9" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="237" t="s">
-        <v>2686</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="237" t="s">
+        <v>2681</v>
+      </c>
+      <c r="B10" s="237" t="s">
+        <v>2728</v>
+      </c>
+      <c r="C10" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="237" t="s">
+        <v>2686</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="237" t="s">
         <v>2683</v>
       </c>
-      <c r="B10" s="237" t="s">
+      <c r="B11" s="237" t="s">
         <v>2729</v>
       </c>
-      <c r="C10" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="237" t="s">
+      <c r="C11" s="237" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="237" t="s">
         <v>2687</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="239" t="s">
+    <row r="12" spans="1:4">
+      <c r="A12" s="239" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="237" t="s">
+      <c r="B12" s="237" t="s">
         <v>2730</v>
       </c>
-      <c r="C11" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="237" t="s">
+      <c r="C12" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="237" t="s">
         <v>2691</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="237" t="s">
-        <v>1872</v>
-      </c>
-      <c r="B12" s="237" t="s">
-        <v>2733</v>
-      </c>
-      <c r="C12" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="237" t="s">
-        <v>2694</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="237" t="s">
-        <v>833</v>
+        <v>1872</v>
       </c>
       <c r="B13" s="237" t="s">
-        <v>2732</v>
+        <v>2733</v>
       </c>
       <c r="C13" s="237" t="s">
         <v>28</v>
       </c>
       <c r="D13" s="237" t="s">
-        <v>2692</v>
+        <v>2694</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="237" t="s">
-        <v>2636</v>
+        <v>833</v>
       </c>
       <c r="B14" s="237" t="s">
-        <v>2735</v>
+        <v>2732</v>
       </c>
       <c r="C14" s="237" t="s">
         <v>28</v>
       </c>
       <c r="D14" s="237" t="s">
-        <v>2640</v>
+        <v>2692</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="237" t="s">
+        <v>2636</v>
+      </c>
+      <c r="B15" s="237" t="s">
+        <v>2735</v>
+      </c>
+      <c r="C15" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="237" t="s">
+        <v>2640</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="237" t="s">
         <v>1090</v>
       </c>
-      <c r="B15" s="237" t="s">
+      <c r="B16" s="237" t="s">
         <v>2736</v>
       </c>
-      <c r="C15" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="237" t="s">
+      <c r="C16" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="237" t="s">
         <v>2644</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="239" t="s">
-        <v>2720</v>
-      </c>
-      <c r="B16" s="239" t="s">
-        <v>2737</v>
-      </c>
-      <c r="C16" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="237" t="s">
-        <v>2655</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="239" t="s">
-        <v>2177</v>
+        <v>2720</v>
       </c>
       <c r="B17" s="239" t="s">
-        <v>2738</v>
+        <v>2737</v>
       </c>
       <c r="C17" s="237" t="s">
         <v>28</v>
@@ -17641,10 +17647,10 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="239" t="s">
-        <v>2721</v>
+        <v>2177</v>
       </c>
       <c r="B18" s="239" t="s">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="C18" s="237" t="s">
         <v>28</v>
@@ -17654,25 +17660,25 @@
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="237" t="s">
-        <v>2656</v>
-      </c>
-      <c r="B19" s="237" t="s">
-        <v>2740</v>
+      <c r="A19" s="239" t="s">
+        <v>2721</v>
+      </c>
+      <c r="B19" s="239" t="s">
+        <v>2739</v>
       </c>
       <c r="C19" s="237" t="s">
         <v>28</v>
       </c>
       <c r="D19" s="237" t="s">
-        <v>2660</v>
+        <v>2655</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="237" t="s">
-        <v>2710</v>
-      </c>
-      <c r="B20" s="238" t="s">
-        <v>2741</v>
+        <v>2656</v>
+      </c>
+      <c r="B20" s="237" t="s">
+        <v>2740</v>
       </c>
       <c r="C20" s="237" t="s">
         <v>28</v>
@@ -17683,38 +17689,38 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="237" t="s">
+        <v>2710</v>
+      </c>
+      <c r="B21" s="238" t="s">
+        <v>2741</v>
+      </c>
+      <c r="C21" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="237" t="s">
+        <v>2660</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="237" t="s">
         <v>2712</v>
       </c>
-      <c r="B21" s="238" t="s">
+      <c r="B22" s="238" t="s">
         <v>2742</v>
       </c>
-      <c r="C21" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="237" t="s">
+      <c r="C22" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="237" t="s">
         <v>2662</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="239" t="s">
-        <v>2663</v>
-      </c>
-      <c r="B22" s="237" t="s">
-        <v>2743</v>
-      </c>
-      <c r="C22" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="237" t="s">
-        <v>2666</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="239" t="s">
-        <v>2722</v>
-      </c>
-      <c r="B23" s="239" t="s">
-        <v>2744</v>
+        <v>2663</v>
+      </c>
+      <c r="B23" s="237" t="s">
+        <v>2743</v>
       </c>
       <c r="C23" s="237" t="s">
         <v>28</v>
@@ -17724,44 +17730,58 @@
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="237" t="s">
-        <v>2718</v>
-      </c>
-      <c r="B24" s="238" t="s">
-        <v>2745</v>
+      <c r="A24" s="239" t="s">
+        <v>2722</v>
+      </c>
+      <c r="B24" s="239" t="s">
+        <v>2744</v>
       </c>
       <c r="C24" s="237" t="s">
         <v>28</v>
       </c>
       <c r="D24" s="237" t="s">
-        <v>2667</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="237" t="s">
+        <v>2718</v>
+      </c>
+      <c r="B25" s="238" t="s">
+        <v>2745</v>
+      </c>
+      <c r="C25" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="237" t="s">
+        <v>2667</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="237" t="s">
         <v>2697</v>
       </c>
-      <c r="B25" s="237" t="s">
+      <c r="B26" s="237" t="s">
         <v>2746</v>
       </c>
-      <c r="C25" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="237" t="s">
+      <c r="C26" s="237" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="237" t="s">
         <v>2089</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="95" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A22" r:id="rId1" display="http://xgin.de/" xr:uid="{6D042F4B-B1B6-714D-834A-FF03BB9AF65F}"/>
-    <hyperlink ref="A11" r:id="rId2" display="http://zprv.de/" xr:uid="{AE8F80AC-32A6-C643-BEE6-694ECBB145F6}"/>
-    <hyperlink ref="A8" r:id="rId3" display="http://iusg.de/" xr:uid="{C28C7857-119A-4744-B0BB-4DDEA3E95E35}"/>
-    <hyperlink ref="B16" r:id="rId4" display="https://finance.yahoo.com/quote/CSBGE3.MI/" xr:uid="{07F4F9CA-E0FA-1C49-87F4-4EBCF7177C7D}"/>
-    <hyperlink ref="B17" r:id="rId5" display="https://finance.yahoo.com/quote/CSBGE7.MI/" xr:uid="{02FC7EA0-25C6-E34E-AB6A-3622B551A50D}"/>
-    <hyperlink ref="B18" r:id="rId6" display="https://finance.yahoo.com/quote/SXRQ.DE/" xr:uid="{4E4D2C26-5E71-C644-AF09-EF7691622628}"/>
-    <hyperlink ref="A23" r:id="rId7" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{6DA783E3-A09C-7C47-88D8-23C14B21E7FE}"/>
-    <hyperlink ref="B23" r:id="rId8" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{894A731F-3358-3D4B-A900-50AD652ED5AE}"/>
+    <hyperlink ref="A23" r:id="rId1" display="http://xgin.de/" xr:uid="{6D042F4B-B1B6-714D-834A-FF03BB9AF65F}"/>
+    <hyperlink ref="A12" r:id="rId2" display="http://zprv.de/" xr:uid="{AE8F80AC-32A6-C643-BEE6-694ECBB145F6}"/>
+    <hyperlink ref="A9" r:id="rId3" display="http://iusg.de/" xr:uid="{C28C7857-119A-4744-B0BB-4DDEA3E95E35}"/>
+    <hyperlink ref="B17" r:id="rId4" display="https://finance.yahoo.com/quote/CSBGE3.MI/" xr:uid="{07F4F9CA-E0FA-1C49-87F4-4EBCF7177C7D}"/>
+    <hyperlink ref="B18" r:id="rId5" display="https://finance.yahoo.com/quote/CSBGE7.MI/" xr:uid="{02FC7EA0-25C6-E34E-AB6A-3622B551A50D}"/>
+    <hyperlink ref="B19" r:id="rId6" display="https://finance.yahoo.com/quote/SXRQ.DE/" xr:uid="{4E4D2C26-5E71-C644-AF09-EF7691622628}"/>
+    <hyperlink ref="A24" r:id="rId7" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{6DA783E3-A09C-7C47-88D8-23C14B21E7FE}"/>
+    <hyperlink ref="B24" r:id="rId8" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{894A731F-3358-3D4B-A900-50AD652ED5AE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Aggiorna TARBIUTH.xlsx con nuovi asset
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TARBIUTH.xlsx
+++ b/TARBIUTH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookpro/Downloads/andcappe_zip/Dashboard/SITO_WEB/Sito personale/portafoglio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9173B583-2356-BF4D-A639-A3BD8687E0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A61BC26-030A-984E-99DA-B34E4B58AD30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4380" yWindow="20" windowWidth="24420" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7570" uniqueCount="2751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7586" uniqueCount="2751">
   <si>
     <t>Simbolo</t>
   </si>
@@ -8582,7 +8582,7 @@
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
   </numFmts>
-  <fonts count="104">
+  <fonts count="106">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -9253,9 +9253,22 @@
       <name val="Abadi"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="8"/>
+      <name val="Abadi"/>
+    </font>
+    <font>
+      <b/>
       <u/>
       <sz val="9"/>
       <color theme="10"/>
+      <name val="Abadi"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Abadi"/>
     </font>
   </fonts>
@@ -9530,7 +9543,7 @@
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="26" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="241">
+  <cellXfs count="246">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -9876,9 +9889,20 @@
     </xf>
     <xf numFmtId="0" fontId="101" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="102" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="103" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="101" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="103" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="103" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="103" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="104" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="105" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="103" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="105" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -9890,7 +9914,75 @@
   <dxfs count="12">
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -9912,74 +10004,6 @@
         <shadow val="0"/>
         <vertAlign val="baseline"/>
         <sz val="9"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color indexed="8"/>
         <name val="Abadi"/>
         <scheme val="none"/>
       </font>
@@ -16269,13 +16293,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D26" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:D26" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D30" totalsRowShown="0" headerRowDxfId="5" dataDxfId="0">
+  <autoFilter ref="A1:D30" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{12AF85F4-CF3E-1A44-9197-52CD700ECF69}" name="SIMBOLO" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{D2DEAFE7-7181-F841-96D9-E16F6CD58118}" name="DESCRIZIONE" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{036B7D95-54D0-CE4A-A97C-6EC741E876E4}" name="VALUTA" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{BC856CD8-BE7C-D246-AFFE-8A0458341DA0}" name="CLASSE" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{12AF85F4-CF3E-1A44-9197-52CD700ECF69}" name="SIMBOLO" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{D2DEAFE7-7181-F841-96D9-E16F6CD58118}" name="DESCRIZIONE" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{036B7D95-54D0-CE4A-A97C-6EC741E876E4}" name="VALUTA" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{BC856CD8-BE7C-D246-AFFE-8A0458341DA0}" name="CLASSE" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -17399,7 +17423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C714FF38-E71E-3648-9A7A-13401C8B9393}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="11"/>
   <cols>
     <col min="1" max="1" width="11.83203125" style="237" customWidth="1"/>
@@ -17422,366 +17446,422 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="235" t="s">
+      <c r="A2" s="239" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="240" t="s">
         <v>2747</v>
       </c>
-      <c r="C2" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="237" t="s">
+      <c r="C2" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="241" t="s">
         <v>2748</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="235" t="s">
+      <c r="A3" s="238" t="s">
+        <v>2571</v>
+      </c>
+      <c r="B3" s="238" t="s">
+        <v>2572</v>
+      </c>
+      <c r="C3" s="243" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="244" t="s">
+        <v>2723</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="241" t="s">
+        <v>2255</v>
+      </c>
+      <c r="B4" s="238" t="s">
+        <v>2614</v>
+      </c>
+      <c r="C4" s="245" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="244" t="s">
+        <v>2723</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="241" t="s">
+        <v>2615</v>
+      </c>
+      <c r="B5" s="238" t="s">
+        <v>2616</v>
+      </c>
+      <c r="C5" s="245" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="244" t="s">
+        <v>2723</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="241" t="s">
+        <v>2617</v>
+      </c>
+      <c r="B6" s="238" t="s">
+        <v>2618</v>
+      </c>
+      <c r="C6" s="245" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="244" t="s">
+        <v>2723</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="239" t="s">
         <v>2619</v>
       </c>
-      <c r="B3" s="238" t="s">
+      <c r="B7" s="238" t="s">
         <v>2724</v>
       </c>
-      <c r="C3" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="237" t="s">
+      <c r="C7" s="241" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="241" t="s">
         <v>2696</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="237" t="s">
+    <row r="8" spans="1:4">
+      <c r="A8" s="241" t="s">
         <v>1091</v>
       </c>
-      <c r="B4" s="238" t="s">
+      <c r="B8" s="238" t="s">
         <v>2734</v>
       </c>
-      <c r="C4" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="237" t="s">
+      <c r="C8" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="241" t="s">
         <v>2635</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="237" t="s">
+    <row r="9" spans="1:4">
+      <c r="A9" s="241" t="s">
         <v>2706</v>
       </c>
-      <c r="B5" s="238" t="s">
+      <c r="B9" s="238" t="s">
         <v>2731</v>
       </c>
-      <c r="C5" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="237" t="s">
+      <c r="C9" s="241" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="241" t="s">
         <v>2708</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15">
-      <c r="A6" s="237" t="s">
+    <row r="10" spans="1:4">
+      <c r="A10" s="241" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="237" t="s">
+      <c r="B10" s="241" t="s">
         <v>2749</v>
       </c>
-      <c r="C6" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="19" t="s">
+      <c r="C10" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="241" t="s">
         <v>2750</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="237" t="s">
+    <row r="11" spans="1:4">
+      <c r="A11" s="241" t="s">
         <v>2668</v>
       </c>
-      <c r="B7" s="237" t="s">
+      <c r="B11" s="241" t="s">
         <v>2725</v>
       </c>
-      <c r="C7" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="237" t="s">
+      <c r="C11" s="241" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="241" t="s">
         <v>2673</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="237" t="s">
+    <row r="12" spans="1:4">
+      <c r="A12" s="241" t="s">
         <v>1089</v>
       </c>
-      <c r="B8" s="237" t="s">
+      <c r="B12" s="241" t="s">
         <v>2726</v>
       </c>
-      <c r="C8" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="237" t="s">
+      <c r="C12" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="241" t="s">
         <v>2680</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="239" t="s">
+    <row r="13" spans="1:4">
+      <c r="A13" s="242" t="s">
         <v>2704</v>
       </c>
-      <c r="B9" s="237" t="s">
+      <c r="B13" s="241" t="s">
         <v>2727</v>
       </c>
-      <c r="C9" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="237" t="s">
+      <c r="C13" s="241" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="241" t="s">
         <v>2685</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="237" t="s">
+    <row r="14" spans="1:4">
+      <c r="A14" s="241" t="s">
         <v>2681</v>
       </c>
-      <c r="B10" s="237" t="s">
+      <c r="B14" s="241" t="s">
         <v>2728</v>
       </c>
-      <c r="C10" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="237" t="s">
+      <c r="C14" s="241" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="241" t="s">
         <v>2686</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="237" t="s">
+    <row r="15" spans="1:4">
+      <c r="A15" s="241" t="s">
         <v>2683</v>
       </c>
-      <c r="B11" s="237" t="s">
+      <c r="B15" s="241" t="s">
         <v>2729</v>
       </c>
-      <c r="C11" s="237" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="237" t="s">
+      <c r="C15" s="241" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="241" t="s">
         <v>2687</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="239" t="s">
+    <row r="16" spans="1:4">
+      <c r="A16" s="242" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="237" t="s">
+      <c r="B16" s="241" t="s">
         <v>2730</v>
       </c>
-      <c r="C12" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="237" t="s">
+      <c r="C16" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="241" t="s">
         <v>2691</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="237" t="s">
+    <row r="17" spans="1:4">
+      <c r="A17" s="241" t="s">
         <v>1872</v>
       </c>
-      <c r="B13" s="237" t="s">
+      <c r="B17" s="241" t="s">
         <v>2733</v>
       </c>
-      <c r="C13" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="237" t="s">
+      <c r="C17" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="241" t="s">
         <v>2694</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="237" t="s">
+    <row r="18" spans="1:4">
+      <c r="A18" s="241" t="s">
         <v>833</v>
       </c>
-      <c r="B14" s="237" t="s">
+      <c r="B18" s="241" t="s">
         <v>2732</v>
       </c>
-      <c r="C14" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="237" t="s">
+      <c r="C18" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="241" t="s">
         <v>2692</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="237" t="s">
+    <row r="19" spans="1:4">
+      <c r="A19" s="241" t="s">
         <v>2636</v>
       </c>
-      <c r="B15" s="237" t="s">
+      <c r="B19" s="241" t="s">
         <v>2735</v>
       </c>
-      <c r="C15" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="237" t="s">
+      <c r="C19" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="241" t="s">
         <v>2640</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="237" t="s">
+    <row r="20" spans="1:4">
+      <c r="A20" s="241" t="s">
         <v>1090</v>
       </c>
-      <c r="B16" s="237" t="s">
+      <c r="B20" s="241" t="s">
         <v>2736</v>
       </c>
-      <c r="C16" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="237" t="s">
+      <c r="C20" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="241" t="s">
         <v>2644</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="239" t="s">
+    <row r="21" spans="1:4">
+      <c r="A21" s="242" t="s">
         <v>2720</v>
       </c>
-      <c r="B17" s="239" t="s">
+      <c r="B21" s="242" t="s">
         <v>2737</v>
       </c>
-      <c r="C17" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="237" t="s">
+      <c r="C21" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="241" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="239" t="s">
+    <row r="22" spans="1:4">
+      <c r="A22" s="242" t="s">
         <v>2177</v>
       </c>
-      <c r="B18" s="239" t="s">
+      <c r="B22" s="242" t="s">
         <v>2738</v>
       </c>
-      <c r="C18" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="237" t="s">
+      <c r="C22" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="241" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="239" t="s">
+    <row r="23" spans="1:4">
+      <c r="A23" s="242" t="s">
         <v>2721</v>
       </c>
-      <c r="B19" s="239" t="s">
+      <c r="B23" s="242" t="s">
         <v>2739</v>
       </c>
-      <c r="C19" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="237" t="s">
+      <c r="C23" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="241" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="237" t="s">
+    <row r="24" spans="1:4">
+      <c r="A24" s="241" t="s">
         <v>2656</v>
       </c>
-      <c r="B20" s="237" t="s">
+      <c r="B24" s="241" t="s">
         <v>2740</v>
       </c>
-      <c r="C20" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="237" t="s">
+      <c r="C24" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="241" t="s">
         <v>2660</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="237" t="s">
+    <row r="25" spans="1:4">
+      <c r="A25" s="241" t="s">
         <v>2710</v>
       </c>
-      <c r="B21" s="238" t="s">
+      <c r="B25" s="238" t="s">
         <v>2741</v>
       </c>
-      <c r="C21" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="237" t="s">
+      <c r="C25" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="241" t="s">
         <v>2660</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="237" t="s">
+    <row r="26" spans="1:4">
+      <c r="A26" s="241" t="s">
         <v>2712</v>
       </c>
-      <c r="B22" s="238" t="s">
+      <c r="B26" s="238" t="s">
         <v>2742</v>
       </c>
-      <c r="C22" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="237" t="s">
+      <c r="C26" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="241" t="s">
         <v>2662</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="239" t="s">
+    <row r="27" spans="1:4">
+      <c r="A27" s="242" t="s">
         <v>2663</v>
       </c>
-      <c r="B23" s="237" t="s">
+      <c r="B27" s="241" t="s">
         <v>2743</v>
       </c>
-      <c r="C23" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="237" t="s">
+      <c r="C27" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" s="241" t="s">
         <v>2666</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="239" t="s">
+    <row r="28" spans="1:4">
+      <c r="A28" s="242" t="s">
         <v>2722</v>
       </c>
-      <c r="B24" s="239" t="s">
+      <c r="B28" s="242" t="s">
         <v>2744</v>
       </c>
-      <c r="C24" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D24" s="237" t="s">
+      <c r="C28" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="241" t="s">
         <v>2666</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="237" t="s">
+    <row r="29" spans="1:4">
+      <c r="A29" s="241" t="s">
         <v>2718</v>
       </c>
-      <c r="B25" s="238" t="s">
+      <c r="B29" s="238" t="s">
         <v>2745</v>
       </c>
-      <c r="C25" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="237" t="s">
+      <c r="C29" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="241" t="s">
         <v>2667</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="237" t="s">
+    <row r="30" spans="1:4">
+      <c r="A30" s="241" t="s">
         <v>2697</v>
       </c>
-      <c r="B26" s="237" t="s">
+      <c r="B30" s="241" t="s">
         <v>2746</v>
       </c>
-      <c r="C26" s="237" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="237" t="s">
+      <c r="C30" s="241" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" s="241" t="s">
         <v>2089</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="95" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A23" r:id="rId1" display="http://xgin.de/" xr:uid="{6D042F4B-B1B6-714D-834A-FF03BB9AF65F}"/>
-    <hyperlink ref="A12" r:id="rId2" display="http://zprv.de/" xr:uid="{AE8F80AC-32A6-C643-BEE6-694ECBB145F6}"/>
-    <hyperlink ref="A9" r:id="rId3" display="http://iusg.de/" xr:uid="{C28C7857-119A-4744-B0BB-4DDEA3E95E35}"/>
-    <hyperlink ref="B17" r:id="rId4" display="https://finance.yahoo.com/quote/CSBGE3.MI/" xr:uid="{07F4F9CA-E0FA-1C49-87F4-4EBCF7177C7D}"/>
-    <hyperlink ref="B18" r:id="rId5" display="https://finance.yahoo.com/quote/CSBGE7.MI/" xr:uid="{02FC7EA0-25C6-E34E-AB6A-3622B551A50D}"/>
-    <hyperlink ref="B19" r:id="rId6" display="https://finance.yahoo.com/quote/SXRQ.DE/" xr:uid="{4E4D2C26-5E71-C644-AF09-EF7691622628}"/>
-    <hyperlink ref="A24" r:id="rId7" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{6DA783E3-A09C-7C47-88D8-23C14B21E7FE}"/>
-    <hyperlink ref="B24" r:id="rId8" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{894A731F-3358-3D4B-A900-50AD652ED5AE}"/>
+    <hyperlink ref="A27" r:id="rId1" display="http://xgin.de/" xr:uid="{6D042F4B-B1B6-714D-834A-FF03BB9AF65F}"/>
+    <hyperlink ref="A16" r:id="rId2" display="http://zprv.de/" xr:uid="{AE8F80AC-32A6-C643-BEE6-694ECBB145F6}"/>
+    <hyperlink ref="A13" r:id="rId3" display="http://iusg.de/" xr:uid="{C28C7857-119A-4744-B0BB-4DDEA3E95E35}"/>
+    <hyperlink ref="B21" r:id="rId4" display="https://finance.yahoo.com/quote/CSBGE3.MI/" xr:uid="{07F4F9CA-E0FA-1C49-87F4-4EBCF7177C7D}"/>
+    <hyperlink ref="B22" r:id="rId5" display="https://finance.yahoo.com/quote/CSBGE7.MI/" xr:uid="{02FC7EA0-25C6-E34E-AB6A-3622B551A50D}"/>
+    <hyperlink ref="B23" r:id="rId6" display="https://finance.yahoo.com/quote/SXRQ.DE/" xr:uid="{4E4D2C26-5E71-C644-AF09-EF7691622628}"/>
+    <hyperlink ref="A28" r:id="rId7" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{6DA783E3-A09C-7C47-88D8-23C14B21E7FE}"/>
+    <hyperlink ref="B28" r:id="rId8" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{894A731F-3358-3D4B-A900-50AD652ED5AE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>